<commit_message>
Upgrade tracker to an Etsy-ready 8-tab template (Ocean & Teal)
Add Cover, How-to, Savings Goals, and Debt Payoff tabs; restyle the whole
workbook in a soft Ocean & Teal aesthetic with a richer 8-card dashboard
(income, savings rate, debt, goals) and three themed charts. Paycheck gains
an annualized column; debt tab adds an APR heat-map. Spec is now generated by
make_spec.py. All 168 formulas verified clean (no #REF!/#DIV/0!), roll-ups
exclude their own total rows, and every chart is palette-themed.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WMQvK9GcdjFML1jvKEoohk
</commit_message>
<xml_diff>
--- a/budget-paycheck-tracker.xlsx
+++ b/budget-paycheck-tracker.xlsx
@@ -7,10 +7,14 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Paycheck" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Budget" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Log" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Dashboard" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Cover" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="How-to" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Paycheck" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Budget" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Log" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Savings Goals" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Debt Payoff" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Dashboard" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,7 +27,7 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="d&quot; &quot;mmm&quot; &quot;yyyy"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,34 +38,44 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="26"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="005A4A42"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="002E4A57"/>
       <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="002E4A3F"/>
-      <sz val="10"/>
+      <color rgb="00FFFFFF"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="002E4A3F"/>
-      <sz val="22"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="002E2A40"/>
-      <sz val="10"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="002E2A40"/>
-      <sz val="22"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="16"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -70,60 +84,48 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002E5E4E"/>
-        <bgColor rgb="002E5E4E"/>
+        <fgColor rgb="00F0EBE1"/>
+        <bgColor rgb="00F0EBE1"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00ECF3F1"/>
-        <bgColor rgb="00ECF3F1"/>
+        <fgColor rgb="002E4A57"/>
+        <bgColor rgb="002E4A57"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FDFBF3"/>
-        <bgColor rgb="00FDFBF3"/>
+        <fgColor rgb="004E9C9C"/>
+        <bgColor rgb="004E9C9C"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F6E5A8"/>
-        <bgColor rgb="00F6E5A8"/>
+        <fgColor rgb="003E7A82"/>
+        <bgColor rgb="003E7A82"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F4C0DB"/>
-        <bgColor rgb="00F4C0DB"/>
+        <fgColor rgb="00EAF3F2"/>
+        <bgColor rgb="00EAF3F2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F8B6C2"/>
-        <bgColor rgb="00F8B6C2"/>
+        <fgColor rgb="00F5F1E8"/>
+        <bgColor rgb="00F5F1E8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="007ED2B6"/>
-        <bgColor rgb="007ED2B6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="0080D2DA"/>
-        <bgColor rgb="0080D2DA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00B9A4E7"/>
-        <bgColor rgb="00B9A4E7"/>
+        <fgColor rgb="005B9AA0"/>
+        <bgColor rgb="005B9AA0"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -133,94 +135,90 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00E8DAD3"/>
+        <color rgb="00CBDCDC"/>
       </left>
       <right style="thin">
-        <color rgb="00E8DAD3"/>
+        <color rgb="00CBDCDC"/>
       </right>
       <top style="thin">
-        <color rgb="00E8DAD3"/>
+        <color rgb="00CBDCDC"/>
       </top>
       <bottom style="thin">
-        <color rgb="00E8DAD3"/>
+        <color rgb="00CBDCDC"/>
       </bottom>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00E8DAD3"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00E8DAD3"/>
-      </right>
-      <top style="thin">
-        <color rgb="00E8DAD3"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00E8DAD3"/>
-      </right>
-      <top style="thin">
-        <color rgb="00E8DAD3"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00E8DAD3"/>
-      </bottom>
-      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -231,8 +229,8 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00FFC7CE"/>
-          <bgColor rgb="00FFC7CE"/>
+          <fgColor rgb="00F4B7B7"/>
+          <bgColor rgb="00F4B7B7"/>
         </patternFill>
       </fill>
     </dxf>
@@ -326,7 +324,7 @@
           </tx>
           <spPr>
             <a:solidFill>
-              <a:srgbClr val="7ED2B6"/>
+              <a:srgbClr val="4E9C9C"/>
             </a:solidFill>
             <a:ln>
               <a:prstDash val="solid"/>
@@ -395,7 +393,7 @@
           </tx>
           <spPr>
             <a:solidFill>
-              <a:srgbClr val="7ED2B6"/>
+              <a:srgbClr val="4E9C9C"/>
             </a:solidFill>
             <a:ln>
               <a:prstDash val="solid"/>
@@ -455,16 +453,113 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Savings Goals'!B1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="4E9C9C"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Savings Goals'!$A$2:$A$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Savings Goals'!$B$2:$B$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Savings Goals'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="A8D0D0"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Savings Goals'!$A$2:$A$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Savings Goals'!$C$2:$C$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>1</col>
+      <col>2</col>
       <colOff>0</colOff>
-      <row>8</row>
+      <row>10</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5760000" cy="2880000"/>
+    <ext cx="6480000" cy="2880000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -481,12 +576,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>1</col>
+      <col>2</col>
       <colOff>0</colOff>
-      <row>23</row>
+      <row>26</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5760000" cy="2880000"/>
+    <ext cx="6480000" cy="2880000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>
@@ -496,6 +591,28 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>42</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6480000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="3" name="Chart 3"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -793,108 +910,134 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="B2:E18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="22" customHeight="1"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="4" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="4" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Amount</t>
-        </is>
-      </c>
-    </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Gross pay (per paycheck)</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="n">
-        <v>2200</v>
-      </c>
+      <c r="B2" s="1" t="n"/>
+      <c r="C2" s="1" t="n"/>
+      <c r="D2" s="1" t="n"/>
+      <c r="E2" s="1" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Federal tax</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="n">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>State tax</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="n">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>FICA (Social Security + Medicare)</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="n">
-        <v>168</v>
-      </c>
-    </row>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>BUDGET  BY  PAYCHECK</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
+    <row r="5"/>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Health insurance</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="n">
-        <v>95</v>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Bi-Weekly Budget &amp; Savings Tracker</t>
+        </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>401(k) retirement</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="n">
-        <v>132</v>
-      </c>
+      <c r="B7" s="1" t="n"/>
+      <c r="C7" s="1" t="n"/>
+      <c r="D7" s="1" t="n"/>
+      <c r="E7" s="1" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Total deductions</t>
-        </is>
-      </c>
-      <c r="B8" s="3">
-        <f>SUM(B3:B7)</f>
-        <v/>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>WHAT'S  INSIDE</t>
+        </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Take-home pay (net)</t>
-        </is>
-      </c>
-      <c r="B9" s="4">
-        <f>B2-B8</f>
-        <v/>
-      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   1  ·  Instructions   —   how to set everything up</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   2  ·  Paycheck   —   your gross pay → take-home</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   3  ·  Budget   —   give every dollar a job</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   4  ·  Paycheck Log   —   track all 26 paydays</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   5  ·  Savings Goals   —   hit every target</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   6  ·  Debt Payoff   —   watch balances shrink</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   7  ·  Dashboard   —   your money at a glance</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="1" t="n"/>
+      <c r="C16" s="1" t="n"/>
+      <c r="D16" s="1" t="n"/>
+      <c r="E16" s="1" t="n"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>♡   Thank you for your purchase   ·   made with care</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="1" t="n"/>
+      <c r="C18" s="1" t="n"/>
+      <c r="D18" s="1" t="n"/>
+      <c r="E18" s="1" t="n"/>
     </row>
   </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="B17:E17"/>
+    <mergeCell ref="B9:E9"/>
+    <mergeCell ref="B8:E8"/>
+    <mergeCell ref="B12:E12"/>
+    <mergeCell ref="B13:E13"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="B15:E15"/>
+    <mergeCell ref="B11:E11"/>
+    <mergeCell ref="B10:E10"/>
+    <mergeCell ref="B3:E5"/>
+    <mergeCell ref="B14:E14"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -905,41 +1048,305 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="92" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>What to do</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>Paycheck tab: enter your gross pay and each deduction. Your take-home pay calculates itself.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Budget tab: set a Budgeted amount per category. Aim to keep 'Left to allocate' at 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Paycheck Log: each payday, type what you Spent. Saved and Cumulative saved fill in for you.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Savings Goals: set a Target for each goal. The progress bar fills as your Saved amount grows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Debt Payoff: enter starting and current balances. Watch '% paid' and total debt move.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Dashboard: open it any time for your take-home, savings rate, debt, and charts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Only the shaded input cells need you — every total, percentage, and chart updates automatically.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>Per paycheck</t>
+        </is>
+      </c>
+      <c r="C1" s="8" t="inlineStr">
+        <is>
+          <t>Per year (×26)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>Gross pay</t>
+        </is>
+      </c>
+      <c r="B2" s="10" t="n">
+        <v>2200</v>
+      </c>
+      <c r="C2" s="10">
+        <f>B2*26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Federal tax</t>
+        </is>
+      </c>
+      <c r="B3" s="11" t="n">
+        <v>264</v>
+      </c>
+      <c r="C3" s="11">
+        <f>B3*26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>State tax</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="n">
+        <v>88</v>
+      </c>
+      <c r="C4" s="10">
+        <f>B4*26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>FICA (Social Security + Medicare)</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="n">
+        <v>168</v>
+      </c>
+      <c r="C5" s="11">
+        <f>B5*26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Health insurance</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="n">
+        <v>95</v>
+      </c>
+      <c r="C6" s="10">
+        <f>B6*26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>401(k) retirement</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="n">
+        <v>132</v>
+      </c>
+      <c r="C7" s="11">
+        <f>B7*26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Total deductions</t>
+        </is>
+      </c>
+      <c r="B8" s="10">
+        <f>SUM(B3:B7)</f>
+        <v/>
+      </c>
+      <c r="C8" s="10">
+        <f>B8*26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Take-home pay (net)</t>
+        </is>
+      </c>
+      <c r="B9" s="11">
+        <f>B2-B8</f>
+        <v/>
+      </c>
+      <c r="C9" s="11">
+        <f>B9*26</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="8" t="inlineStr">
         <is>
           <t>Budgeted</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="8" t="inlineStr">
         <is>
           <t>% of take-home</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="9" t="inlineStr">
         <is>
           <t>Rent / housing</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n">
+      <c r="B2" s="10" t="n">
         <v>600</v>
       </c>
-      <c r="C2" s="5">
+      <c r="C2" s="12">
         <f>IF($B$13=0,0,B2/$B$13)</f>
         <v/>
       </c>
@@ -950,24 +1357,24 @@
           <t>Utilities</t>
         </is>
       </c>
-      <c r="B3" s="4" t="n">
+      <c r="B3" s="11" t="n">
         <v>90</v>
       </c>
-      <c r="C3" s="6">
+      <c r="C3" s="13">
         <f>IF($B$13=0,0,B3/$B$13)</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>Groceries</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n">
+      <c r="B4" s="10" t="n">
         <v>220</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="12">
         <f>IF($B$13=0,0,B4/$B$13)</f>
         <v/>
       </c>
@@ -978,24 +1385,24 @@
           <t>Transportation / gas</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" s="11" t="n">
         <v>100</v>
       </c>
-      <c r="C5" s="6">
+      <c r="C5" s="13">
         <f>IF($B$13=0,0,B5/$B$13)</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>Phone + internet</t>
         </is>
       </c>
-      <c r="B6" s="3" t="n">
+      <c r="B6" s="10" t="n">
         <v>60</v>
       </c>
-      <c r="C6" s="5">
+      <c r="C6" s="12">
         <f>IF($B$13=0,0,B6/$B$13)</f>
         <v/>
       </c>
@@ -1006,24 +1413,24 @@
           <t>Subscriptions</t>
         </is>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B7" s="11" t="n">
         <v>30</v>
       </c>
-      <c r="C7" s="6">
+      <c r="C7" s="13">
         <f>IF($B$13=0,0,B7/$B$13)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>Debt payment</t>
         </is>
       </c>
-      <c r="B8" s="3" t="n">
+      <c r="B8" s="10" t="n">
         <v>100</v>
       </c>
-      <c r="C8" s="5">
+      <c r="C8" s="12">
         <f>IF($B$13=0,0,B8/$B$13)</f>
         <v/>
       </c>
@@ -1034,24 +1441,24 @@
           <t>Savings</t>
         </is>
       </c>
-      <c r="B9" s="4" t="n">
+      <c r="B9" s="11" t="n">
         <v>150</v>
       </c>
-      <c r="C9" s="6">
+      <c r="C9" s="13">
         <f>IF($B$13=0,0,B9/$B$13)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>Fun / dining out</t>
         </is>
       </c>
-      <c r="B10" s="3" t="n">
+      <c r="B10" s="10" t="n">
         <v>60</v>
       </c>
-      <c r="C10" s="5">
+      <c r="C10" s="12">
         <f>IF($B$13=0,0,B10/$B$13)</f>
         <v/>
       </c>
@@ -1062,25 +1469,25 @@
           <t>Miscellaneous</t>
         </is>
       </c>
-      <c r="B11" s="4" t="n">
+      <c r="B11" s="11" t="n">
         <v>43</v>
       </c>
-      <c r="C11" s="6">
+      <c r="C11" s="13">
         <f>IF($B$13=0,0,B11/$B$13)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>Total budgeted</t>
         </is>
       </c>
-      <c r="B12" s="3">
+      <c r="B12" s="10">
         <f>SUM(B2:B11)</f>
         <v/>
       </c>
-      <c r="C12" s="5">
+      <c r="C12" s="12">
         <f>IF($B$13=0,0,B12/$B$13)</f>
         <v/>
       </c>
@@ -1091,22 +1498,22 @@
           <t>Take-home pay (net)</t>
         </is>
       </c>
-      <c r="B13" s="4">
+      <c r="B13" s="11">
         <f>Paycheck!B9</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>Left to allocate</t>
         </is>
       </c>
-      <c r="B14" s="3">
+      <c r="B14" s="10">
         <f>B13-B12</f>
         <v/>
       </c>
-      <c r="C14" s="2" t="n"/>
+      <c r="C14" s="9" t="n"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="C2:C11">
@@ -1114,7 +1521,7 @@
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="007ED2B6"/>
+        <color rgb="004E9C9C"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -1127,7 +1534,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1145,57 +1552,57 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="8" t="inlineStr">
         <is>
           <t>Pay date</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="8" t="inlineStr">
         <is>
           <t>Net pay</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="8" t="inlineStr">
         <is>
           <t>Spent</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="8" t="inlineStr">
         <is>
           <t>Saved</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="8" t="inlineStr">
         <is>
           <t>Cumulative saved</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="7">
+      <c r="B2" s="14">
         <f>DATE(2026,1,2)+14*(2-2)</f>
         <v/>
       </c>
-      <c r="C2" s="3">
+      <c r="C2" s="10">
         <f>Paycheck!$B$9</f>
         <v/>
       </c>
-      <c r="D2" s="3" t="n">
+      <c r="D2" s="10" t="n">
         <v>1303</v>
       </c>
-      <c r="E2" s="3">
+      <c r="E2" s="10">
         <f>C2-D2</f>
         <v/>
       </c>
-      <c r="F2" s="3">
+      <c r="F2" s="10">
         <f>SUM($E$2:E2)</f>
         <v/>
       </c>
@@ -1204,46 +1611,46 @@
       <c r="A3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="8">
+      <c r="B3" s="15">
         <f>DATE(2026,1,2)+14*(3-2)</f>
         <v/>
       </c>
-      <c r="C3" s="4">
+      <c r="C3" s="11">
         <f>Paycheck!$B$9</f>
         <v/>
       </c>
-      <c r="D3" s="4" t="n">
+      <c r="D3" s="11" t="n">
         <v>1303</v>
       </c>
-      <c r="E3" s="4">
+      <c r="E3" s="11">
         <f>C3-D3</f>
         <v/>
       </c>
-      <c r="F3" s="4">
+      <c r="F3" s="11">
         <f>SUM($E$2:E3)</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="7">
+      <c r="B4" s="14">
         <f>DATE(2026,1,2)+14*(4-2)</f>
         <v/>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="10">
         <f>Paycheck!$B$9</f>
         <v/>
       </c>
-      <c r="D4" s="3" t="n">
+      <c r="D4" s="10" t="n">
         <v>1303</v>
       </c>
-      <c r="E4" s="3">
+      <c r="E4" s="10">
         <f>C4-D4</f>
         <v/>
       </c>
-      <c r="F4" s="3">
+      <c r="F4" s="10">
         <f>SUM($E$2:E4)</f>
         <v/>
       </c>
@@ -1252,46 +1659,46 @@
       <c r="A5" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="8">
+      <c r="B5" s="15">
         <f>DATE(2026,1,2)+14*(5-2)</f>
         <v/>
       </c>
-      <c r="C5" s="4">
+      <c r="C5" s="11">
         <f>Paycheck!$B$9</f>
         <v/>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D5" s="11" t="n">
         <v>1303</v>
       </c>
-      <c r="E5" s="4">
+      <c r="E5" s="11">
         <f>C5-D5</f>
         <v/>
       </c>
-      <c r="F5" s="4">
+      <c r="F5" s="11">
         <f>SUM($E$2:E5)</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="7">
+      <c r="B6" s="14">
         <f>DATE(2026,1,2)+14*(6-2)</f>
         <v/>
       </c>
-      <c r="C6" s="3">
+      <c r="C6" s="10">
         <f>Paycheck!$B$9</f>
         <v/>
       </c>
-      <c r="D6" s="3" t="n">
+      <c r="D6" s="10" t="n">
         <v>1303</v>
       </c>
-      <c r="E6" s="3">
+      <c r="E6" s="10">
         <f>C6-D6</f>
         <v/>
       </c>
-      <c r="F6" s="3">
+      <c r="F6" s="10">
         <f>SUM($E$2:E6)</f>
         <v/>
       </c>
@@ -1300,46 +1707,46 @@
       <c r="A7" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="8">
+      <c r="B7" s="15">
         <f>DATE(2026,1,2)+14*(7-2)</f>
         <v/>
       </c>
-      <c r="C7" s="4">
+      <c r="C7" s="11">
         <f>Paycheck!$B$9</f>
         <v/>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="D7" s="11" t="n">
         <v>1303</v>
       </c>
-      <c r="E7" s="4">
+      <c r="E7" s="11">
         <f>C7-D7</f>
         <v/>
       </c>
-      <c r="F7" s="4">
+      <c r="F7" s="11">
         <f>SUM($E$2:E7)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="7">
+      <c r="B8" s="14">
         <f>DATE(2026,1,2)+14*(8-2)</f>
         <v/>
       </c>
-      <c r="C8" s="3">
+      <c r="C8" s="10">
         <f>Paycheck!$B$9</f>
         <v/>
       </c>
-      <c r="D8" s="3" t="n">
+      <c r="D8" s="10" t="n">
         <v>1303</v>
       </c>
-      <c r="E8" s="3">
+      <c r="E8" s="10">
         <f>C8-D8</f>
         <v/>
       </c>
-      <c r="F8" s="3">
+      <c r="F8" s="10">
         <f>SUM($E$2:E8)</f>
         <v/>
       </c>
@@ -1348,46 +1755,46 @@
       <c r="A9" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="8">
+      <c r="B9" s="15">
         <f>DATE(2026,1,2)+14*(9-2)</f>
         <v/>
       </c>
-      <c r="C9" s="4">
+      <c r="C9" s="11">
         <f>Paycheck!$B$9</f>
         <v/>
       </c>
-      <c r="D9" s="4" t="n">
+      <c r="D9" s="11" t="n">
         <v>1303</v>
       </c>
-      <c r="E9" s="4">
+      <c r="E9" s="11">
         <f>C9-D9</f>
         <v/>
       </c>
-      <c r="F9" s="4">
+      <c r="F9" s="11">
         <f>SUM($E$2:E9)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
+      <c r="A10" s="9" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="7">
+      <c r="B10" s="14">
         <f>DATE(2026,1,2)+14*(10-2)</f>
         <v/>
       </c>
-      <c r="C10" s="3">
+      <c r="C10" s="10">
         <f>Paycheck!$B$9</f>
         <v/>
       </c>
-      <c r="D10" s="3" t="n">
+      <c r="D10" s="10" t="n">
         <v>1303</v>
       </c>
-      <c r="E10" s="3">
+      <c r="E10" s="10">
         <f>C10-D10</f>
         <v/>
       </c>
-      <c r="F10" s="3">
+      <c r="F10" s="10">
         <f>SUM($E$2:E10)</f>
         <v/>
       </c>
@@ -1396,46 +1803,46 @@
       <c r="A11" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="8">
+      <c r="B11" s="15">
         <f>DATE(2026,1,2)+14*(11-2)</f>
         <v/>
       </c>
-      <c r="C11" s="4">
+      <c r="C11" s="11">
         <f>Paycheck!$B$9</f>
         <v/>
       </c>
-      <c r="D11" s="4" t="n">
+      <c r="D11" s="11" t="n">
         <v>1303</v>
       </c>
-      <c r="E11" s="4">
+      <c r="E11" s="11">
         <f>C11-D11</f>
         <v/>
       </c>
-      <c r="F11" s="4">
+      <c r="F11" s="11">
         <f>SUM($E$2:E11)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n">
+      <c r="A12" s="9" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="7">
+      <c r="B12" s="14">
         <f>DATE(2026,1,2)+14*(12-2)</f>
         <v/>
       </c>
-      <c r="C12" s="3">
+      <c r="C12" s="10">
         <f>Paycheck!$B$9</f>
         <v/>
       </c>
-      <c r="D12" s="3" t="n">
+      <c r="D12" s="10" t="n">
         <v>1303</v>
       </c>
-      <c r="E12" s="3">
+      <c r="E12" s="10">
         <f>C12-D12</f>
         <v/>
       </c>
-      <c r="F12" s="3">
+      <c r="F12" s="10">
         <f>SUM($E$2:E12)</f>
         <v/>
       </c>
@@ -1444,46 +1851,46 @@
       <c r="A13" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="8">
+      <c r="B13" s="15">
         <f>DATE(2026,1,2)+14*(13-2)</f>
         <v/>
       </c>
-      <c r="C13" s="4">
+      <c r="C13" s="11">
         <f>Paycheck!$B$9</f>
         <v/>
       </c>
-      <c r="D13" s="4" t="n">
+      <c r="D13" s="11" t="n">
         <v>1303</v>
       </c>
-      <c r="E13" s="4">
+      <c r="E13" s="11">
         <f>C13-D13</f>
         <v/>
       </c>
-      <c r="F13" s="4">
+      <c r="F13" s="11">
         <f>SUM($E$2:E13)</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n">
+      <c r="A14" s="9" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="7">
+      <c r="B14" s="14">
         <f>DATE(2026,1,2)+14*(14-2)</f>
         <v/>
       </c>
-      <c r="C14" s="3">
+      <c r="C14" s="10">
         <f>Paycheck!$B$9</f>
         <v/>
       </c>
-      <c r="D14" s="3" t="n">
+      <c r="D14" s="10" t="n">
         <v>1303</v>
       </c>
-      <c r="E14" s="3">
+      <c r="E14" s="10">
         <f>C14-D14</f>
         <v/>
       </c>
-      <c r="F14" s="3">
+      <c r="F14" s="10">
         <f>SUM($E$2:E14)</f>
         <v/>
       </c>
@@ -1492,46 +1899,46 @@
       <c r="A15" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="8">
+      <c r="B15" s="15">
         <f>DATE(2026,1,2)+14*(15-2)</f>
         <v/>
       </c>
-      <c r="C15" s="4">
+      <c r="C15" s="11">
         <f>Paycheck!$B$9</f>
         <v/>
       </c>
-      <c r="D15" s="4" t="n">
+      <c r="D15" s="11" t="n">
         <v>1303</v>
       </c>
-      <c r="E15" s="4">
+      <c r="E15" s="11">
         <f>C15-D15</f>
         <v/>
       </c>
-      <c r="F15" s="4">
+      <c r="F15" s="11">
         <f>SUM($E$2:E15)</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n">
+      <c r="A16" s="9" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="7">
+      <c r="B16" s="14">
         <f>DATE(2026,1,2)+14*(16-2)</f>
         <v/>
       </c>
-      <c r="C16" s="3">
+      <c r="C16" s="10">
         <f>Paycheck!$B$9</f>
         <v/>
       </c>
-      <c r="D16" s="3" t="n">
+      <c r="D16" s="10" t="n">
         <v>1303</v>
       </c>
-      <c r="E16" s="3">
+      <c r="E16" s="10">
         <f>C16-D16</f>
         <v/>
       </c>
-      <c r="F16" s="3">
+      <c r="F16" s="10">
         <f>SUM($E$2:E16)</f>
         <v/>
       </c>
@@ -1540,46 +1947,46 @@
       <c r="A17" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="8">
+      <c r="B17" s="15">
         <f>DATE(2026,1,2)+14*(17-2)</f>
         <v/>
       </c>
-      <c r="C17" s="4">
+      <c r="C17" s="11">
         <f>Paycheck!$B$9</f>
         <v/>
       </c>
-      <c r="D17" s="4" t="n">
+      <c r="D17" s="11" t="n">
         <v>1303</v>
       </c>
-      <c r="E17" s="4">
+      <c r="E17" s="11">
         <f>C17-D17</f>
         <v/>
       </c>
-      <c r="F17" s="4">
+      <c r="F17" s="11">
         <f>SUM($E$2:E17)</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="n">
+      <c r="A18" s="9" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="7">
+      <c r="B18" s="14">
         <f>DATE(2026,1,2)+14*(18-2)</f>
         <v/>
       </c>
-      <c r="C18" s="3">
+      <c r="C18" s="10">
         <f>Paycheck!$B$9</f>
         <v/>
       </c>
-      <c r="D18" s="3" t="n">
+      <c r="D18" s="10" t="n">
         <v>1303</v>
       </c>
-      <c r="E18" s="3">
+      <c r="E18" s="10">
         <f>C18-D18</f>
         <v/>
       </c>
-      <c r="F18" s="3">
+      <c r="F18" s="10">
         <f>SUM($E$2:E18)</f>
         <v/>
       </c>
@@ -1588,46 +1995,46 @@
       <c r="A19" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="8">
+      <c r="B19" s="15">
         <f>DATE(2026,1,2)+14*(19-2)</f>
         <v/>
       </c>
-      <c r="C19" s="4">
+      <c r="C19" s="11">
         <f>Paycheck!$B$9</f>
         <v/>
       </c>
-      <c r="D19" s="4" t="n">
+      <c r="D19" s="11" t="n">
         <v>1303</v>
       </c>
-      <c r="E19" s="4">
+      <c r="E19" s="11">
         <f>C19-D19</f>
         <v/>
       </c>
-      <c r="F19" s="4">
+      <c r="F19" s="11">
         <f>SUM($E$2:E19)</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="n">
+      <c r="A20" s="9" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="7">
+      <c r="B20" s="14">
         <f>DATE(2026,1,2)+14*(20-2)</f>
         <v/>
       </c>
-      <c r="C20" s="3">
+      <c r="C20" s="10">
         <f>Paycheck!$B$9</f>
         <v/>
       </c>
-      <c r="D20" s="3" t="n">
+      <c r="D20" s="10" t="n">
         <v>1303</v>
       </c>
-      <c r="E20" s="3">
+      <c r="E20" s="10">
         <f>C20-D20</f>
         <v/>
       </c>
-      <c r="F20" s="3">
+      <c r="F20" s="10">
         <f>SUM($E$2:E20)</f>
         <v/>
       </c>
@@ -1636,46 +2043,46 @@
       <c r="A21" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="8">
+      <c r="B21" s="15">
         <f>DATE(2026,1,2)+14*(21-2)</f>
         <v/>
       </c>
-      <c r="C21" s="4">
+      <c r="C21" s="11">
         <f>Paycheck!$B$9</f>
         <v/>
       </c>
-      <c r="D21" s="4" t="n">
+      <c r="D21" s="11" t="n">
         <v>1303</v>
       </c>
-      <c r="E21" s="4">
+      <c r="E21" s="11">
         <f>C21-D21</f>
         <v/>
       </c>
-      <c r="F21" s="4">
+      <c r="F21" s="11">
         <f>SUM($E$2:E21)</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="n">
+      <c r="A22" s="9" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="7">
+      <c r="B22" s="14">
         <f>DATE(2026,1,2)+14*(22-2)</f>
         <v/>
       </c>
-      <c r="C22" s="3">
+      <c r="C22" s="10">
         <f>Paycheck!$B$9</f>
         <v/>
       </c>
-      <c r="D22" s="3" t="n">
+      <c r="D22" s="10" t="n">
         <v>1303</v>
       </c>
-      <c r="E22" s="3">
+      <c r="E22" s="10">
         <f>C22-D22</f>
         <v/>
       </c>
-      <c r="F22" s="3">
+      <c r="F22" s="10">
         <f>SUM($E$2:E22)</f>
         <v/>
       </c>
@@ -1684,46 +2091,46 @@
       <c r="A23" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="8">
+      <c r="B23" s="15">
         <f>DATE(2026,1,2)+14*(23-2)</f>
         <v/>
       </c>
-      <c r="C23" s="4">
+      <c r="C23" s="11">
         <f>Paycheck!$B$9</f>
         <v/>
       </c>
-      <c r="D23" s="4" t="n">
+      <c r="D23" s="11" t="n">
         <v>1303</v>
       </c>
-      <c r="E23" s="4">
+      <c r="E23" s="11">
         <f>C23-D23</f>
         <v/>
       </c>
-      <c r="F23" s="4">
+      <c r="F23" s="11">
         <f>SUM($E$2:E23)</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n">
+      <c r="A24" s="9" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="7">
+      <c r="B24" s="14">
         <f>DATE(2026,1,2)+14*(24-2)</f>
         <v/>
       </c>
-      <c r="C24" s="3">
+      <c r="C24" s="10">
         <f>Paycheck!$B$9</f>
         <v/>
       </c>
-      <c r="D24" s="3" t="n">
+      <c r="D24" s="10" t="n">
         <v>1303</v>
       </c>
-      <c r="E24" s="3">
+      <c r="E24" s="10">
         <f>C24-D24</f>
         <v/>
       </c>
-      <c r="F24" s="3">
+      <c r="F24" s="10">
         <f>SUM($E$2:E24)</f>
         <v/>
       </c>
@@ -1732,46 +2139,46 @@
       <c r="A25" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="8">
+      <c r="B25" s="15">
         <f>DATE(2026,1,2)+14*(25-2)</f>
         <v/>
       </c>
-      <c r="C25" s="4">
+      <c r="C25" s="11">
         <f>Paycheck!$B$9</f>
         <v/>
       </c>
-      <c r="D25" s="4" t="n">
+      <c r="D25" s="11" t="n">
         <v>1303</v>
       </c>
-      <c r="E25" s="4">
+      <c r="E25" s="11">
         <f>C25-D25</f>
         <v/>
       </c>
-      <c r="F25" s="4">
+      <c r="F25" s="11">
         <f>SUM($E$2:E25)</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="n">
+      <c r="A26" s="9" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="7">
+      <c r="B26" s="14">
         <f>DATE(2026,1,2)+14*(26-2)</f>
         <v/>
       </c>
-      <c r="C26" s="3">
+      <c r="C26" s="10">
         <f>Paycheck!$B$9</f>
         <v/>
       </c>
-      <c r="D26" s="3" t="n">
+      <c r="D26" s="10" t="n">
         <v>1303</v>
       </c>
-      <c r="E26" s="3">
+      <c r="E26" s="10">
         <f>C26-D26</f>
         <v/>
       </c>
-      <c r="F26" s="3">
+      <c r="F26" s="10">
         <f>SUM($E$2:E26)</f>
         <v/>
       </c>
@@ -1780,22 +2187,22 @@
       <c r="A27" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="8">
+      <c r="B27" s="15">
         <f>DATE(2026,1,2)+14*(27-2)</f>
         <v/>
       </c>
-      <c r="C27" s="4">
+      <c r="C27" s="11">
         <f>Paycheck!$B$9</f>
         <v/>
       </c>
-      <c r="D27" s="4" t="n">
+      <c r="D27" s="11" t="n">
         <v>1303</v>
       </c>
-      <c r="E27" s="4">
+      <c r="E27" s="11">
         <f>C27-D27</f>
         <v/>
       </c>
-      <c r="F27" s="4">
+      <c r="F27" s="11">
         <f>SUM($E$2:E27)</f>
         <v/>
       </c>
@@ -1807,9 +2214,9 @@
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
         <cfvo type="max"/>
-        <color rgb="00FDFBF3"/>
-        <color rgb="0099E4EB"/>
-        <color rgb="007ED2B6"/>
+        <color rgb="00F0EBE1"/>
+        <color rgb="00A8D0D0"/>
+        <color rgb="004E9C9C"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -1817,110 +2224,615 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:G23"/>
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Goal</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
+      <c r="C1" s="8" t="inlineStr">
+        <is>
+          <t>Saved</t>
+        </is>
+      </c>
+      <c r="D1" s="8" t="inlineStr">
+        <is>
+          <t>Remaining</t>
+        </is>
+      </c>
+      <c r="E1" s="8" t="inlineStr">
+        <is>
+          <t>% Complete</t>
+        </is>
+      </c>
+      <c r="F1" s="8" t="inlineStr">
+        <is>
+          <t>Target date</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>Emergency fund</t>
+        </is>
+      </c>
+      <c r="B2" s="10" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C2" s="10" t="n">
+        <v>1500</v>
+      </c>
+      <c r="D2" s="10">
+        <f>MAX(B2-C2,0)</f>
+        <v/>
+      </c>
+      <c r="E2" s="12">
+        <f>IF(B2=0,0,C2/B2)</f>
+        <v/>
+      </c>
+      <c r="F2" s="14">
+        <f>DATE(2026,12,31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Vacation</t>
+        </is>
+      </c>
+      <c r="B3" s="11" t="n">
+        <v>2500</v>
+      </c>
+      <c r="C3" s="11" t="n">
+        <v>800</v>
+      </c>
+      <c r="D3" s="11">
+        <f>MAX(B3-C3,0)</f>
+        <v/>
+      </c>
+      <c r="E3" s="13">
+        <f>IF(B3=0,0,C3/B3)</f>
+        <v/>
+      </c>
+      <c r="F3" s="15">
+        <f>DATE(2026,8,15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>New car fund</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="n">
+        <v>8000</v>
+      </c>
+      <c r="C4" s="10" t="n">
+        <v>2200</v>
+      </c>
+      <c r="D4" s="10">
+        <f>MAX(B4-C4,0)</f>
+        <v/>
+      </c>
+      <c r="E4" s="12">
+        <f>IF(B4=0,0,C4/B4)</f>
+        <v/>
+      </c>
+      <c r="F4" s="14">
+        <f>DATE(2027,6,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Holiday gifts</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="n">
+        <v>1200</v>
+      </c>
+      <c r="C5" s="11" t="n">
+        <v>300</v>
+      </c>
+      <c r="D5" s="11">
+        <f>MAX(B5-C5,0)</f>
+        <v/>
+      </c>
+      <c r="E5" s="13">
+        <f>IF(B5=0,0,C5/B5)</f>
+        <v/>
+      </c>
+      <c r="F5" s="15">
+        <f>DATE(2026,12,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Home down payment</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="n">
+        <v>20000</v>
+      </c>
+      <c r="C6" s="10" t="n">
+        <v>4500</v>
+      </c>
+      <c r="D6" s="10">
+        <f>MAX(B6-C6,0)</f>
+        <v/>
+      </c>
+      <c r="E6" s="12">
+        <f>IF(B6=0,0,C6/B6)</f>
+        <v/>
+      </c>
+      <c r="F6" s="14">
+        <f>DATE(2028,1,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B7" s="11">
+        <f>SUM(B2:B6)</f>
+        <v/>
+      </c>
+      <c r="C7" s="11">
+        <f>SUM(C2:C6)</f>
+        <v/>
+      </c>
+      <c r="D7" s="11">
+        <f>SUM(D2:D6)</f>
+        <v/>
+      </c>
+      <c r="E7" s="13">
+        <f>IF(B7=0,0,C7/B7)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="E2:E6">
+    <cfRule type="dataBar" priority="1">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="004E9C9C"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Debt</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>Starting balance</t>
+        </is>
+      </c>
+      <c r="C1" s="8" t="inlineStr">
+        <is>
+          <t>Current balance</t>
+        </is>
+      </c>
+      <c r="D1" s="8" t="inlineStr">
+        <is>
+          <t>Paid off</t>
+        </is>
+      </c>
+      <c r="E1" s="8" t="inlineStr">
+        <is>
+          <t>% paid</t>
+        </is>
+      </c>
+      <c r="F1" s="8" t="inlineStr">
+        <is>
+          <t>APR</t>
+        </is>
+      </c>
+      <c r="G1" s="8" t="inlineStr">
+        <is>
+          <t>Min payment</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>Credit card</t>
+        </is>
+      </c>
+      <c r="B2" s="10" t="n">
+        <v>4200</v>
+      </c>
+      <c r="C2" s="10" t="n">
+        <v>3100</v>
+      </c>
+      <c r="D2" s="10">
+        <f>B2-C2</f>
+        <v/>
+      </c>
+      <c r="E2" s="12">
+        <f>IF(B2=0,0,D2/B2)</f>
+        <v/>
+      </c>
+      <c r="F2" s="16" t="n">
+        <v>0.1999</v>
+      </c>
+      <c r="G2" s="10" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Car loan</t>
+        </is>
+      </c>
+      <c r="B3" s="11" t="n">
+        <v>18000</v>
+      </c>
+      <c r="C3" s="11" t="n">
+        <v>11500</v>
+      </c>
+      <c r="D3" s="11">
+        <f>B3-C3</f>
+        <v/>
+      </c>
+      <c r="E3" s="13">
+        <f>IF(B3=0,0,D3/B3)</f>
+        <v/>
+      </c>
+      <c r="F3" s="17" t="n">
+        <v>0.0549</v>
+      </c>
+      <c r="G3" s="11" t="n">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>Student loan</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="n">
+        <v>24000</v>
+      </c>
+      <c r="C4" s="10" t="n">
+        <v>15800</v>
+      </c>
+      <c r="D4" s="10">
+        <f>B4-C4</f>
+        <v/>
+      </c>
+      <c r="E4" s="12">
+        <f>IF(B4=0,0,D4/B4)</f>
+        <v/>
+      </c>
+      <c r="F4" s="16" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="G4" s="10" t="n">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Personal loan</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="n">
+        <v>6000</v>
+      </c>
+      <c r="C5" s="11" t="n">
+        <v>2400</v>
+      </c>
+      <c r="D5" s="11">
+        <f>B5-C5</f>
+        <v/>
+      </c>
+      <c r="E5" s="13">
+        <f>IF(B5=0,0,D5/B5)</f>
+        <v/>
+      </c>
+      <c r="F5" s="17" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="G5" s="11" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B6" s="10">
+        <f>SUM(B2:B5)</f>
+        <v/>
+      </c>
+      <c r="C6" s="10">
+        <f>SUM(C2:C5)</f>
+        <v/>
+      </c>
+      <c r="D6" s="10">
+        <f>SUM(D2:D5)</f>
+        <v/>
+      </c>
+      <c r="E6" s="12">
+        <f>IF(B6=0,0,D6/B6)</f>
+        <v/>
+      </c>
+      <c r="F6" s="9" t="n"/>
+      <c r="G6" s="10">
+        <f>SUM(G2:G5)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="E2:E5">
+    <cfRule type="dataBar" priority="1">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="004E9C9C"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F2:F5">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="007ED2B6"/>
+        <color rgb="00F6E5A8"/>
+        <color rgb="00E8A6A6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="C2:I42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="18" customHeight="1"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="3.1" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="3.1" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="3.1" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="3" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="3" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="3" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
     <col width="3" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="3" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="2">
-      <c r="B2" s="9" t="inlineStr">
-        <is>
-          <t>P A Y C H E C K   O V E R V I E W</t>
+      <c r="C2" s="18" t="inlineStr">
+        <is>
+          <t>M O N E Y   A T   A   G L A N C E</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="10" t="n"/>
-      <c r="C3" s="10" t="n"/>
-      <c r="D3" s="10" t="n"/>
-      <c r="E3" s="10" t="n"/>
-      <c r="F3" s="10" t="n"/>
-      <c r="G3" s="10" t="n"/>
+      <c r="C3" s="19" t="n"/>
+      <c r="D3" s="19" t="n"/>
+      <c r="E3" s="19" t="n"/>
+      <c r="F3" s="19" t="n"/>
+      <c r="G3" s="19" t="n"/>
+      <c r="H3" s="19" t="n"/>
+      <c r="I3" s="19" t="n"/>
     </row>
     <row r="4">
-      <c r="B4" s="11" t="inlineStr">
+      <c r="C4" s="20" t="inlineStr">
         <is>
           <t>Take-home / paycheck</t>
         </is>
       </c>
-      <c r="C4" s="12" t="n"/>
-      <c r="D4" s="13" t="inlineStr">
-        <is>
-          <t>Saved per year</t>
-        </is>
-      </c>
-      <c r="E4" s="12" t="n"/>
-      <c r="F4" s="14" t="inlineStr">
+      <c r="D4" s="19" t="n"/>
+      <c r="E4" s="21" t="inlineStr">
+        <is>
+          <t>Avg monthly income</t>
+        </is>
+      </c>
+      <c r="F4" s="19" t="n"/>
+      <c r="G4" s="22" t="inlineStr">
+        <is>
+          <t>Saved / year</t>
+        </is>
+      </c>
+      <c r="H4" s="19" t="n"/>
+      <c r="I4" s="21" t="inlineStr">
         <is>
           <t>Savings rate</t>
         </is>
       </c>
-      <c r="G4" s="12" t="n"/>
     </row>
     <row r="5">
-      <c r="B5" s="15">
+      <c r="C5" s="23">
         <f>Paycheck!B9</f>
         <v/>
       </c>
-      <c r="C5" s="12" t="n"/>
-      <c r="D5" s="16">
+      <c r="D5" s="19" t="n"/>
+      <c r="E5" s="24">
+        <f>Paycheck!B9*26/12</f>
+        <v/>
+      </c>
+      <c r="F5" s="19" t="n"/>
+      <c r="G5" s="25">
         <f>SUM(Log!E2:E27)</f>
         <v/>
       </c>
-      <c r="E5" s="12" t="n"/>
-      <c r="F5" s="17">
+      <c r="H5" s="19" t="n"/>
+      <c r="I5" s="26">
         <f>IF(SUM(Log!C2:C27)=0,0,SUM(Log!E2:E27)/SUM(Log!C2:C27))</f>
         <v/>
       </c>
-      <c r="G5" s="12" t="n"/>
     </row>
     <row r="6">
-      <c r="B6" s="10" t="n"/>
-      <c r="C6" s="10" t="n"/>
-      <c r="D6" s="10" t="n"/>
-      <c r="E6" s="10" t="n"/>
-      <c r="F6" s="10" t="n"/>
-      <c r="G6" s="10" t="n"/>
+      <c r="C6" s="19" t="n"/>
+      <c r="D6" s="19" t="n"/>
+      <c r="E6" s="19" t="n"/>
+      <c r="F6" s="19" t="n"/>
+      <c r="G6" s="19" t="n"/>
+      <c r="H6" s="19" t="n"/>
+      <c r="I6" s="19" t="n"/>
+    </row>
+    <row r="7">
+      <c r="C7" s="21" t="inlineStr">
+        <is>
+          <t>Total saved (goals)</t>
+        </is>
+      </c>
+      <c r="D7" s="19" t="n"/>
+      <c r="E7" s="22" t="inlineStr">
+        <is>
+          <t>Goals progress</t>
+        </is>
+      </c>
+      <c r="F7" s="19" t="n"/>
+      <c r="G7" s="20" t="inlineStr">
+        <is>
+          <t>Total debt left</t>
+        </is>
+      </c>
+      <c r="H7" s="19" t="n"/>
+      <c r="I7" s="21" t="inlineStr">
+        <is>
+          <t>Debt paid off</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="B8" s="18" t="inlineStr">
+      <c r="C8" s="24">
+        <f>SUM('Savings Goals'!C2:C6)</f>
+        <v/>
+      </c>
+      <c r="D8" s="19" t="n"/>
+      <c r="E8" s="27">
+        <f>IF(SUM('Savings Goals'!B2:B6)=0,0,SUM('Savings Goals'!C2:C6)/SUM('Savings Goals'!B2:B6))</f>
+        <v/>
+      </c>
+      <c r="F8" s="19" t="n"/>
+      <c r="G8" s="23">
+        <f>SUM('Debt Payoff'!C2:C5)</f>
+        <v/>
+      </c>
+      <c r="H8" s="19" t="n"/>
+      <c r="I8" s="24">
+        <f>SUM('Debt Payoff'!D2:D5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="C10" s="28" t="inlineStr">
         <is>
           <t>B U D G E T   B Y   C A T E G O R Y</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="B23" s="19" t="inlineStr">
-        <is>
-          <t>C U M U L A T I V E   S A V I N G S   ·   26   P A Y C H E C K S</t>
+    <row r="26">
+      <c r="C26" s="29" t="inlineStr">
+        <is>
+          <t>S A V I N G S   G R O W T H   ·   26   P A Y C H E C K S</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="C42" s="30" t="inlineStr">
+        <is>
+          <t>G O A L S   ·   T A R G E T   vs   S A V E D</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B23:G23"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="B8:G8"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="B4:C4"/>
+  <mergeCells count="20">
+    <mergeCell ref="I5"/>
+    <mergeCell ref="C8"/>
+    <mergeCell ref="I8"/>
+    <mergeCell ref="G4"/>
+    <mergeCell ref="I4"/>
+    <mergeCell ref="C7"/>
+    <mergeCell ref="E7"/>
+    <mergeCell ref="C42:I42"/>
+    <mergeCell ref="C5"/>
+    <mergeCell ref="E5"/>
+    <mergeCell ref="E8"/>
+    <mergeCell ref="C4"/>
+    <mergeCell ref="G8"/>
+    <mergeCell ref="C26:I26"/>
+    <mergeCell ref="E4"/>
+    <mergeCell ref="G7"/>
+    <mergeCell ref="I7"/>
+    <mergeCell ref="C10:I10"/>
+    <mergeCell ref="C2:I2"/>
+    <mergeCell ref="G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>